<commit_message>
Retrait de fr-CA dans les formats de date, bouton Ouvrir le PDF, note sur le groupe de sécurité
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -185,7 +185,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ChecklistTI" displayName="ChecklistTI" ref="A1:D10" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ChecklistTI" displayName="ChecklistTI" ref="A1:D11" headerRowCount="1">
   <autoFilter ref="A1:D10"/>
   <tableColumns count="4">
     <tableColumn id="1" name="N°"/>
@@ -1112,7 +1112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1261,7 +1261,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Partager l'application avec les gestionnaires (rôle Utilisateur).</t>
+          <t>Groupe de sécurité de l'environnement : y inclure tous les utilisateurs de l'application (personnes évaluées et gestionnaires) et les testeurs ; sinon « You are not a member of the environment's security group ».</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1277,15 +1277,30 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
+          <t>Partager l'application avec les gestionnaires (rôle Utilisateur).</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Tests du guide (partie 8) en pré-prod, puis répéter en prod.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Annie + TI</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Mise à jour du 28 octobre : PDF joint au dossier (une version), PDF du plan, écran allégé, Transmis aux RH, dates sans fr-CA ; documents à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -789,7 +789,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>35 colonnes (guide étape 3.2). TypeRencontre = Choix, « Cases à cocher (autoriser plusieurs sélections) ». Index : Annee, Statut, CourrielPersonne, CourrielSI, CourrielSH, CourrielDirecteur (PAS TypeRencontre). Versions : Oui.</t>
+          <t>35 colonnes (guide étape 3.2). TypeRencontre = Choix, « Cases à cocher (autoriser plusieurs sélections) ». Index : Annee, Statut, CourrielPersonne, CourrielSI, CourrielSH, CourrielDirecteur (PAS TypeRencontre). Versions : Oui. Pièces jointes : Activé.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -833,22 +833,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Bibliothèque de documents</t>
+          <t>Pièces jointes de la liste Appreciations</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Appreciations_PDF</t>
+          <t>(aucune bibliothèque)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Aucune colonne à ajouter.</t>
+          <t>Pièces jointes activées sur la liste Appreciations (réglage par défaut). Le flux 3 y joint le PDF complet et le PDF du plan, en remplaçant l'ancienne version.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Héritage arrêté : Propriétaires = Contrôle total ; RH – Appréciations = Lecture. Retirer Membres et Visiteurs. Le flux 3 donne l'accès PDF par PDF.</t>
+          <t>Mêmes accès que le dossier (personnes du dossier + RH).</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Déclencheur : Power Apps (V2) — bouton Aperçu PDF</t>
+          <t>Déclencheur : Power Apps (V2) — boutons Aperçu PDF et Créer le PDF du plan ; joint le PDF au dossier</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Créer sur le site cible : liste Appreciations, liste Parametres, bibliothèque Appreciations_PDF, groupe RH – Appréciations (onglet SharePoint).</t>
+          <t>Créer sur le site cible : liste Appreciations (pièces jointes activées), liste Parametres, groupe RH – Appréciations (onglet SharePoint).</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Retrait des onglets Synthèse et Plan de développement et du PDF du plan ; documents à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -843,7 +843,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Pièces jointes activées sur la liste Appreciations (réglage par défaut). Le flux 3 y joint le PDF complet et le PDF du plan, en remplaçant l'ancienne version.</t>
+          <t>Pièces jointes activées sur la liste Appreciations (réglage par défaut). Le flux 3 y joint le PDF complet, en remplaçant l'ancienne version.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Déclencheur : Power Apps (V2) — boutons Aperçu PDF et Créer le PDF du plan ; joint le PDF au dossier</t>
+          <t>Déclencheur : Power Apps (V2) — bouton Aperçu PDF ; joint le PDF au dossier (une seule version)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Appréciation de la contribution : version finale (28 octobre 2026)
Tous les documents, visuels, Excel et présentation portent la mention
version finale ; ajout d'une archive ZIP regroupant les livrables.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SharePoint" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solution" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist TI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="À propos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SharePoint" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solution" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist TI" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +32,16 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0000285E"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00009E49"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -66,6 +77,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,6 +500,129 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Appréciation de la contribution — fichier de déploiement</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>VERSION FINALE — 28 octobre 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Onglet</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Contenu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Variables</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Les 5 variables d'environnement : noms exacts et valeurs pour le développement, la pré-prod et la prod</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SharePoint</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Listes, groupe et autorisations à créer sur chaque site (le PDF est joint à chaque dossier : aucune bibliothèque)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Solution</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Composants de la solution : application, 3 flux, 4 références de connexion, 5 variables</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Checklist TI</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Étapes d'import et de vérification pour les TI (pré-prod, puis prod)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Responsable</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Annie Audet, Ressources humaines (RH-SST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Documents liés</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>GUIDE-MISE-EN-PRODUCTION.docx · FLUX-FINAUX.txt · DOSSIER-AUTORISATION-TI.docx</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -728,7 +865,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -914,7 +1051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1106,7 +1243,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Correction du type de rencontre et paquet de transmission PréProd pour les TI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="À propos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SharePoint" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solution" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist TI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenu du ZIP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testeurs PréProd" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Variables" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SharePoint" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Solution" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist TI" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -500,7 +502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -517,13 +519,11 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>VERSION FINALE — 28 octobre 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-    </row>
+          <t>VERSION FINALE — 28 octobre 2026 · mise à jour du 29 octobre (transmission PréProd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -585,30 +585,54 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
-      <c r="B9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Contenu du ZIP</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Les fichiers remis aux TI pour la PréProd, et à quoi sert chacun</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Testeurs PréProd</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Les personnes à ajouter au groupe de sécurité de l'environnement PréProd et au site SharePoint</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Annie Audet, Ressources humaines (RH-SST)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Documents liés</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>GUIDE-MISE-EN-PRODUCTION.docx · FLUX-FINAUX.txt · DOSSIER-AUTORISATION-TI.docx</t>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>BORDEREAU-TRANSMISSION-TI.docx · GUIDE-MISE-EN-PRODUCTION.docx · DOSSIER-AUTORISATION-TI.docx · FLUX-FINAUX.txt</t>
         </is>
       </c>
     </row>
@@ -618,6 +642,311 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Fichier</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>À quoi il sert</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Dans le ZIP ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Solution-ApplicationAppreciation_1_0_0_2_managed.zip</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Solution gérée à importer (application, 3 flux, 5 variables, 4 références de connexion)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>À AJOUTER par Annie (export Power Apps)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>BORDEREAU-TRANSMISSION-TI.docx</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Lisez-moi : contenu du paquet, ordre des étapes, personne-ressource</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>DOSSIER-AUTORISATION-TI.docx</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Réponses au formulaire de mise en PréProd (texte « Commentaires », testeurs, renseignements personnels)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>GUIDE-MISE-EN-PRODUCTION.docx</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Guide technique : SharePoint (partie 4), flux (partie 6), tests (partie 8), remise (partie 9)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Variables-environnement-et-deploiement.xlsx</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Ce fichier : variables, SharePoint, composants, checklist, testeurs</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>FLUX-FINAUX.txt</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Les 3 flux, action par action (référence en cas de vérification)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Schema-solution.jpg</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Schéma d'ensemble de la solution</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Courriel</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Rôle de test</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Groupe de sécurité PréProd (✓)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Membres du site SharePoint PréProd (✓)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Béland, Véronique (RH-RSI)</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Personne en appréciation / supérieure (paire)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Ajouter chaque testeur au groupe de sécurité de l'environnement PréProd ET au groupe Membres du site SharePoint PréProd. Sans le groupe de sécurité : « You are not a member of the environment's security group ».</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A11:E12"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -865,7 +1194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1051,7 +1380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1243,13 +1572,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1286,7 +1615,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Créer sur le site cible : liste Appreciations (pièces jointes activées), liste Parametres, groupe RH – Appréciations (onglet SharePoint).</t>
+          <t>Créer sur le site cible les listes Appreciations et Parametres avec « Nouveau › Liste › À partir d'une liste existante » (listes du bac à sable : colonnes identiques), puis appliquer les réglages de l'onglet SharePoint (index, pièces jointes, versions, autorisations) et créer le groupe RH – Appréciations.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1398,7 +1727,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Groupe de sécurité de l'environnement : y inclure tous les utilisateurs de l'application (personnes évaluées et gestionnaires) et les testeurs ; sinon « You are not a member of the environment's security group ».</t>
+          <t>Groupe de sécurité de l'environnement : y inclure les testeurs (onglet Testeurs PréProd) ; en prod, tous les utilisateurs (personnes évaluées et gestionnaires). Sinon : « You are not a member of the environment's security group ».</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1436,6 +1765,21 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>Annie + TI</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ajouter les testeurs au groupe Membres du site SharePoint PréProd (onglet Testeurs PréProd).</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Demande aux TI : déploiement pour le 9 novembre, revue de l'application et des groupes de sécurité
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -523,7 +523,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -647,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -704,12 +703,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>BORDEREAU-TRANSMISSION-TI.docx</t>
+          <t>DEMANDE-TI-DEPLOIEMENT-9-NOVEMBRE.docx</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Lisez-moi : contenu du paquet, ordre des étapes, personne-ressource</t>
+          <t>La demande : PréProd/Prod, revue de l'application, groupes de sécurité, recommandations, échéancier du 9 novembre</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -724,12 +723,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>DOSSIER-AUTORISATION-TI.docx</t>
+          <t>BORDEREAU-TRANSMISSION-TI.docx</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Réponses au formulaire de mise en PréProd (texte « Commentaires », testeurs, renseignements personnels)</t>
+          <t>Lisez-moi : contenu du paquet, ordre des étapes, personne-ressource</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -744,12 +743,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>GUIDE-MISE-EN-PRODUCTION.docx</t>
+          <t>DOSSIER-AUTORISATION-TI.docx</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Guide technique : SharePoint (partie 4), flux (partie 6), tests (partie 8), remise (partie 9)</t>
+          <t>Réponses au formulaire de mise en PréProd (texte « Commentaires », testeurs, renseignements personnels)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -764,12 +763,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Variables-environnement-et-deploiement.xlsx</t>
+          <t>GUIDE-MISE-EN-PRODUCTION.docx</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Ce fichier : variables, SharePoint, composants, checklist, testeurs</t>
+          <t>Guide technique : SharePoint (partie 4), flux (partie 6), tests (partie 8), remise (partie 9)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -784,12 +783,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>FLUX-FINAUX.txt</t>
+          <t>Variables-environnement-et-deploiement.xlsx</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Les 3 flux, action par action (référence en cas de vérification)</t>
+          <t>Ce fichier : variables, SharePoint, composants, checklist, testeurs</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -804,15 +803,35 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>FLUX-FINAUX.txt</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Les 3 flux, action par action (référence en cas de vérification)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>Schema-solution.jpg</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Schéma d'ensemble de la solution</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>

</xml_diff>

<commit_message>
Section B : échelle des postures de leadership à 4 niveaux, avec la note 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -519,10 +519,11 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>VERSION FINALE — 28 octobre 2026 · mise à jour du 29 octobre (transmission PréProd)</t>
-        </is>
-      </c>
-    </row>
+          <t>VERSION FINALE — 28 octobre 2026 · mises à jour du 29 et du 30 octobre (transmission PréProd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -683,7 +684,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Solution-ApplicationAppreciation_1_0_0_2_managed.zip</t>
+          <t>Solution-ApplicationAppreciation_1_0_0_3_managed.zip</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -949,6 +950,7 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
PréProd et conformité aux exigences des TI : guide, formules, flux, documents pour Documents TI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -519,11 +519,10 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>VERSION FINALE — 28 octobre 2026 · mises à jour du 29 et du 30 octobre (transmission PréProd)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>VERSION FINALE — 28 octobre 2026 · mises à jour du 29 et du 30 octobre (conformité TI, solution 1.0.0.4)</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -684,7 +683,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Solution-ApplicationAppreciation_1_0_0_3_managed.zip</t>
+          <t>Solution-ApplicationAppreciation_1_0_0_4_managed.zip</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -950,7 +949,6 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -973,7 +971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1025,7 +1023,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Site Appréciations</t>
+          <t>APCONT_SiteWeb-RHSST-AppreciationContribution</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1040,7 +1038,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>parameters('Site Appréciations (rhdsst_SiteApprciations)')</t>
+          <t>parameters('APCONT_SiteWeb-RHSST-AppreciationContribution (rhdsst_SiteApprciations)')</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1050,7 +1048,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>(site de pré-prod, à fournir par les TI)</t>
+          <t>[adresse du site PréProd]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1062,7 +1060,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Liste Appreciations</t>
+          <t>APCONT_Appreciations</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1077,7 +1075,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>parameters('Liste Appreciations (rhdsst_ListeAppreciations)')</t>
+          <t>parameters('APCONT_Appreciations (rhdsst_ListeAppreciations)')</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1087,19 +1085,19 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>liste Appreciations (à choisir sur le site de pré-prod)</t>
+          <t>liste APCONT_Appreciations (site PréProd)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>liste Appreciations (à choisir sur le site de prod)</t>
+          <t>liste APCONT_Appreciations (site Prod)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Liste Parametres</t>
+          <t>APCONT_Parametres</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1114,7 +1112,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>parameters('Liste Parametres (rhdsst_ListeParametres)')</t>
+          <t>parameters('APCONT_Parametres (rhdsst_ListeParametres)')</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1124,19 +1122,19 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>liste Parametres (site de pré-prod)</t>
+          <t>liste APCONT_Parametres (site PréProd)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>liste Parametres (site de prod)</t>
+          <t>liste APCONT_Parametres (site Prod)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Courriel paie</t>
+          <t>APCONT_CourrielPaie</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1151,7 +1149,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>parameters('Courriel paie (rhdsst_Courrielpaie)')</t>
+          <t>parameters('APCONT_CourrielPaie (rhdsst_Courrielpaie)')</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1173,7 +1171,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lienapplication</t>
+          <t>APCONT_LienApplication</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1188,7 +1186,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>parameters('Lienapplication (rhdsst_Lienapplication)')</t>
+          <t>parameters('APCONT_LienApplication (rhdsst_Lienapplication)')</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1204,6 +1202,50 @@
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>lien web de l'application après import en prod</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>APCONT_CourrielSoutien</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>rhdsst_APCONT_CourrielSoutien (à vérifier)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Texte</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>parameters('APCONT_CourrielSoutien (rhdsst_APCONT_CourrielSoutien)')</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>annie.audet@ville.quebec.qc.ca</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>[adresse du soutien]</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>[adresse du soutien]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Toutes les variables : section Avancé › bascule d'export de la valeur à NON (la valeur n'est pas exportée).</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1313,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Appreciations</t>
+          <t>APCONT_Appreciations</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1281,7 +1323,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Héritage arrêté : Propriétaires = Contrôle total ; RH – Appréciations = Lecture ; Membres du site = Collaboration. Aucune personne seule, aucun autre groupe.</t>
+          <t>Héritage arrêté : Propriétaires = Contrôle total ; APCONT_RH = Lecture ; APCONT_Utilisateurs (groupe local contenant G-IS-APP-xxxxx) = Collaboration ; Membres et Visiteurs retirés. Aucune personne seule, aucun autre groupe.</t>
         </is>
       </c>
     </row>
@@ -1298,7 +1340,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Parametres</t>
+          <t>APCONT_Parametres</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1352,7 +1394,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>RH – Appréciations</t>
+          <t>APCONT_RH</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1636,7 +1678,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Créer sur le site cible les listes Appreciations et Parametres avec « Nouveau › Liste › À partir d'une liste existante » (listes du bac à sable : colonnes identiques), puis appliquer les réglages de l'onglet SharePoint (index, pièces jointes, versions, autorisations) et créer le groupe RH – Appréciations.</t>
+          <t>Créer sur le site cible les listes APCONT_Appreciations et APCONT_Parametres (« Nouveau › Liste › À partir d'une liste existante »), les groupes locaux APCONT_Utilisateurs (contient G-IS-APP-xxxxx) et APCONT_RH sans droit sur le site, puis les autorisations des listes (guide PréProd, partie A).</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Site PréProd « RH Power Apps Données PréProd » et réponse sur le site de données Prod
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -523,6 +523,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -949,6 +950,7 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
+    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1048,12 +1050,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[adresse du site PréProd]</t>
+          <t>RH Power Apps Données PréProd ([adresse URL])</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>(site officiel, à fournir par les TI)</t>
+          <t>site de données Prod des TI ([à confirmer])</t>
         </is>
       </c>
     </row>
@@ -1242,6 +1244,7 @@
         </is>
       </c>
     </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Acronyme SRHVQ, pas à pas du site PréProd, analyse de la solution et du risque OneDrive
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -1025,7 +1025,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>APCONT_SiteWeb-RHSST-AppreciationContribution</t>
+          <t>SRHVQ_SiteWeb-RHSST-AppreciationContribution</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_SiteWeb-RHSST-AppreciationContribution (rhdsst_SiteApprciations)')</t>
+          <t>parameters('SRHVQ_SiteWeb-RHSST-AppreciationContribution (rhdsst_SiteApprciations)')</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1062,7 +1062,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>APCONT_Appreciations</t>
+          <t>SRHVQ_Appreciations</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -1077,7 +1077,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_Appreciations (rhdsst_ListeAppreciations)')</t>
+          <t>parameters('SRHVQ_Appreciations (rhdsst_ListeAppreciations)')</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1087,19 +1087,19 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>liste APCONT_Appreciations (site PréProd)</t>
+          <t>liste SRHVQ_Appreciations (site PréProd)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>liste APCONT_Appreciations (site Prod)</t>
+          <t>liste SRHVQ_Appreciations (site Prod)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>APCONT_Parametres</t>
+          <t>SRHVQ_Parametres</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_Parametres (rhdsst_ListeParametres)')</t>
+          <t>parameters('SRHVQ_Parametres (rhdsst_ListeParametres)')</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1124,19 +1124,19 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>liste APCONT_Parametres (site PréProd)</t>
+          <t>liste SRHVQ_Parametres (site PréProd)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>liste APCONT_Parametres (site Prod)</t>
+          <t>liste SRHVQ_Parametres (site Prod)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>APCONT_CourrielPaie</t>
+          <t>SRHVQ_CourrielPaie</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1151,7 +1151,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_CourrielPaie (rhdsst_Courrielpaie)')</t>
+          <t>parameters('SRHVQ_CourrielPaie (rhdsst_Courrielpaie)')</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1173,7 +1173,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>APCONT_LienApplication</t>
+          <t>SRHVQ_LienApplication</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_LienApplication (rhdsst_Lienapplication)')</t>
+          <t>parameters('SRHVQ_LienApplication (rhdsst_Lienapplication)')</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1210,12 +1210,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>APCONT_CourrielSoutien</t>
+          <t>SRHVQ_CourrielSoutien</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>rhdsst_APCONT_CourrielSoutien (à vérifier)</t>
+          <t>rhdsst_SRHVQ_CourrielSoutien (à vérifier)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>parameters('APCONT_CourrielSoutien (rhdsst_APCONT_CourrielSoutien)')</t>
+          <t>parameters('SRHVQ_CourrielSoutien (rhdsst_SRHVQ_CourrielSoutien)')</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1316,7 +1316,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>APCONT_Appreciations</t>
+          <t>SRHVQ_Appreciations</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Héritage arrêté : Propriétaires = Contrôle total ; APCONT_RH = Lecture ; APCONT_Utilisateurs (groupe local contenant G-IS-APP-xxxxx) = Collaboration ; Membres et Visiteurs retirés. Aucune personne seule, aucun autre groupe.</t>
+          <t>Héritage arrêté : Propriétaires = Contrôle total ; SRHVQ_RH = Lecture ; SRHVQ_Utilisateurs (groupe local contenant G-IS-APP-xxxxx) = Collaboration ; Membres et Visiteurs retirés. Aucune personne seule, aucun autre groupe.</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>APCONT_Parametres</t>
+          <t>SRHVQ_Parametres</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>APCONT_RH</t>
+          <t>SRHVQ_RH</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Créer sur le site cible les listes APCONT_Appreciations et APCONT_Parametres (« Nouveau › Liste › À partir d'une liste existante »), les groupes locaux APCONT_Utilisateurs (contient G-IS-APP-xxxxx) et APCONT_RH sans droit sur le site, puis les autorisations des listes (guide PréProd, partie A).</t>
+          <t>Créer sur le site cible les listes SRHVQ_Appreciations et SRHVQ_Parametres (« Nouveau › Liste › À partir d'une liste existante »), les groupes locaux SRHVQ_Utilisateurs (contient G-IS-APP-xxxxx) et SRHVQ_RH sans droit sur le site, puis les autorisations des listes (guide PréProd, partie A).</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Solution : 6 références de connexion documentées pour les TI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FRdAzq8p3F9gJJe5MA3G79
</commit_message>
<xml_diff>
--- a/powerapps/Variables-environnement-et-deploiement.xlsx
+++ b/powerapps/Variables-environnement-et-deploiement.xlsx
@@ -523,7 +523,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -950,7 +949,6 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr"/>
     </row>
-    <row r="10"/>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1244,7 +1242,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1452,7 +1449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1553,7 +1550,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SharePoint Appreciation</t>
+          <t>SharePoint Appreciations</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1570,12 +1567,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Utilisateurs Office 365 Appreciations</t>
+          <t>Outlook Appreciations</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Application (nom dans l'application : Utilisateursd’Office365)</t>
+          <t>Flux 2, courriels d'erreur</t>
         </is>
       </c>
     </row>
@@ -1587,12 +1584,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Outlook Appreciations</t>
+          <t>Utilisateurs Office 365 Appreciations</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Flux 2</t>
+          <t>Application</t>
         </is>
       </c>
     </row>
@@ -1604,27 +1601,61 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>OneDrive Appreciations</t>
+          <t>OneDrive Entreprise RHDSSTDAAT-1b68d</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Flux 3 (NOUVEAU — conversion en PDF)</t>
+          <t>Flux 3 (conversion PDF) — compte de service avec OneDrive initialisé</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Référence de connexion</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>SharePoint RHDSSTDAAT-11da3</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Ancienne référence, gardée par sécurité (actions SharePoint possibles du flux 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Référence de connexion</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Office 365 Outlook Gestion_formulaire_approb…</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Ancienne référence, gardée par sécurité (actions Outlook possibles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Variables d'environnement</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>5 variables</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>6 variables (SRHVQ_…)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Voir l'onglet Variables</t>
         </is>
@@ -1729,7 +1760,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Références de connexion : choisir les connexions du compte de service (4 références, dont OneDrive Appreciations).</t>
+          <t>Références de connexion : choisir les connexions du compte de service pour les 6 références (onglet Solution). Le compte de service doit avoir un OneDrive initialisé.</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">

</xml_diff>